<commit_message>
Add initial dataset file with sample data for analysis
</commit_message>
<xml_diff>
--- a/public/Dataset.xlsx
+++ b/public/Dataset.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1169">
   <si>
     <t>No</t>
   </si>
@@ -3486,6 +3486,42 @@
   </si>
   <si>
     <t>2026-04-25 07:45:00</t>
+  </si>
+  <si>
+    <t>SIKC16953855555</t>
+  </si>
+  <si>
+    <t>IKC202309666666</t>
+  </si>
+  <si>
+    <t>2026-05-02 01:53:00</t>
+  </si>
+  <si>
+    <t>2026-05-18 01:53:00</t>
+  </si>
+  <si>
+    <t>SIKC169538577777</t>
+  </si>
+  <si>
+    <t>IKC20237777777</t>
+  </si>
+  <si>
+    <t>2026-04-05 01:56:00</t>
+  </si>
+  <si>
+    <t>2026-04-08 01:56:00</t>
+  </si>
+  <si>
+    <t>SIKC169354666666</t>
+  </si>
+  <si>
+    <t>IKC20230666666</t>
+  </si>
+  <si>
+    <t>2026-04-18 02:09:00</t>
+  </si>
+  <si>
+    <t>2026-04-04 02:09:00</t>
   </si>
 </sst>
 </file>
@@ -3825,7 +3861,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:AE280"/>
+  <dimension ref="A1:AE283"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:31">
@@ -25958,6 +25994,243 @@
       </c>
       <c r="AE280">
         <v>123123123.0</v>
+      </c>
+    </row>
+    <row r="281" spans="1:31">
+      <c r="A281">
+        <v>280</v>
+      </c>
+      <c r="B281" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C281" t="s">
+        <v>1158</v>
+      </c>
+      <c r="D281" t="s">
+        <v>1159</v>
+      </c>
+      <c r="E281" t="s">
+        <v>1160</v>
+      </c>
+      <c r="F281" t="s">
+        <v>35</v>
+      </c>
+      <c r="G281"/>
+      <c r="H281" t="s">
+        <v>36</v>
+      </c>
+      <c r="I281" t="s">
+        <v>35</v>
+      </c>
+      <c r="J281" t="s">
+        <v>37</v>
+      </c>
+      <c r="K281" t="s">
+        <v>38</v>
+      </c>
+      <c r="L281" t="s">
+        <v>38</v>
+      </c>
+      <c r="M281" t="s">
+        <v>38</v>
+      </c>
+      <c r="N281" t="s">
+        <v>38</v>
+      </c>
+      <c r="O281" t="s">
+        <v>38</v>
+      </c>
+      <c r="P281" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q281" t="s">
+        <v>39</v>
+      </c>
+      <c r="R281" t="s">
+        <v>39</v>
+      </c>
+      <c r="S281" t="s">
+        <v>39</v>
+      </c>
+      <c r="T281" t="s">
+        <v>1143</v>
+      </c>
+      <c r="U281" t="s">
+        <v>39</v>
+      </c>
+      <c r="V281"/>
+      <c r="W281"/>
+      <c r="X281"/>
+      <c r="Y281"/>
+      <c r="Z281"/>
+      <c r="AA281"/>
+      <c r="AB281"/>
+      <c r="AC281">
+        <v>0.0</v>
+      </c>
+      <c r="AD281">
+        <v>6665757.0</v>
+      </c>
+      <c r="AE281">
+        <v>6665757.0</v>
+      </c>
+    </row>
+    <row r="282" spans="1:31">
+      <c r="A282">
+        <v>281</v>
+      </c>
+      <c r="B282" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C282" t="s">
+        <v>1162</v>
+      </c>
+      <c r="D282" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E282" t="s">
+        <v>1164</v>
+      </c>
+      <c r="F282" t="s">
+        <v>35</v>
+      </c>
+      <c r="G282"/>
+      <c r="H282" t="s">
+        <v>1137</v>
+      </c>
+      <c r="I282" t="s">
+        <v>35</v>
+      </c>
+      <c r="J282" t="s">
+        <v>37</v>
+      </c>
+      <c r="K282" t="s">
+        <v>38</v>
+      </c>
+      <c r="L282" t="s">
+        <v>38</v>
+      </c>
+      <c r="M282" t="s">
+        <v>38</v>
+      </c>
+      <c r="N282" t="s">
+        <v>38</v>
+      </c>
+      <c r="O282" t="s">
+        <v>38</v>
+      </c>
+      <c r="P282" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q282" t="s">
+        <v>39</v>
+      </c>
+      <c r="R282" t="s">
+        <v>39</v>
+      </c>
+      <c r="S282" t="s">
+        <v>39</v>
+      </c>
+      <c r="T282" t="s">
+        <v>45</v>
+      </c>
+      <c r="U282" t="s">
+        <v>39</v>
+      </c>
+      <c r="V282"/>
+      <c r="W282"/>
+      <c r="X282"/>
+      <c r="Y282"/>
+      <c r="Z282"/>
+      <c r="AA282"/>
+      <c r="AB282"/>
+      <c r="AC282">
+        <v>0.0</v>
+      </c>
+      <c r="AD282">
+        <v>66666666.0</v>
+      </c>
+      <c r="AE282">
+        <v>66666666.0</v>
+      </c>
+    </row>
+    <row r="283" spans="1:31">
+      <c r="A283">
+        <v>282</v>
+      </c>
+      <c r="B283" t="s">
+        <v>1165</v>
+      </c>
+      <c r="C283" t="s">
+        <v>1166</v>
+      </c>
+      <c r="D283" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E283" t="s">
+        <v>1168</v>
+      </c>
+      <c r="F283" t="s">
+        <v>35</v>
+      </c>
+      <c r="G283"/>
+      <c r="H283" t="s">
+        <v>36</v>
+      </c>
+      <c r="I283" t="s">
+        <v>35</v>
+      </c>
+      <c r="J283" t="s">
+        <v>37</v>
+      </c>
+      <c r="K283" t="s">
+        <v>38</v>
+      </c>
+      <c r="L283" t="s">
+        <v>38</v>
+      </c>
+      <c r="M283" t="s">
+        <v>38</v>
+      </c>
+      <c r="N283" t="s">
+        <v>38</v>
+      </c>
+      <c r="O283" t="s">
+        <v>38</v>
+      </c>
+      <c r="P283" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q283" t="s">
+        <v>39</v>
+      </c>
+      <c r="R283" t="s">
+        <v>39</v>
+      </c>
+      <c r="S283" t="s">
+        <v>39</v>
+      </c>
+      <c r="T283" t="s">
+        <v>1138</v>
+      </c>
+      <c r="U283" t="s">
+        <v>39</v>
+      </c>
+      <c r="V283"/>
+      <c r="W283"/>
+      <c r="X283"/>
+      <c r="Y283"/>
+      <c r="Z283"/>
+      <c r="AA283"/>
+      <c r="AB283"/>
+      <c r="AC283">
+        <v>0.0</v>
+      </c>
+      <c r="AD283">
+        <v>65656565.0</v>
+      </c>
+      <c r="AE283">
+        <v>65656565.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add full documentation for automateCRM system covering architecture, features, Docker setup, CI/CD, and Excel integration
</commit_message>
<xml_diff>
--- a/public/Dataset.xlsx
+++ b/public/Dataset.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1178">
   <si>
     <t>No</t>
   </si>
@@ -3522,6 +3522,33 @@
   </si>
   <si>
     <t>2026-04-04 02:09:00</t>
+  </si>
+  <si>
+    <t>SIKC16953833333</t>
+  </si>
+  <si>
+    <t>IKC20230933333</t>
+  </si>
+  <si>
+    <t>2026-04-16 02:14:00</t>
+  </si>
+  <si>
+    <t>2026-04-04 02:14:00</t>
+  </si>
+  <si>
+    <t>Transfer</t>
+  </si>
+  <si>
+    <t>SIKC1693500000</t>
+  </si>
+  <si>
+    <t>IKC20230900000</t>
+  </si>
+  <si>
+    <t>2026-04-06 02:15:00</t>
+  </si>
+  <si>
+    <t>2026-04-25 02:15:00</t>
   </si>
 </sst>
 </file>
@@ -3861,7 +3888,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:AE283"/>
+  <dimension ref="A1:AE285"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:31">
@@ -26231,6 +26258,162 @@
       </c>
       <c r="AE283">
         <v>65656565.0</v>
+      </c>
+    </row>
+    <row r="284" spans="1:31">
+      <c r="A284">
+        <v>283</v>
+      </c>
+      <c r="B284" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C284" t="s">
+        <v>1170</v>
+      </c>
+      <c r="D284" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E284" t="s">
+        <v>1172</v>
+      </c>
+      <c r="F284" t="s">
+        <v>35</v>
+      </c>
+      <c r="G284"/>
+      <c r="H284"/>
+      <c r="I284" t="s">
+        <v>35</v>
+      </c>
+      <c r="J284" t="s">
+        <v>37</v>
+      </c>
+      <c r="K284" t="s">
+        <v>38</v>
+      </c>
+      <c r="L284" t="s">
+        <v>38</v>
+      </c>
+      <c r="M284" t="s">
+        <v>38</v>
+      </c>
+      <c r="N284" t="s">
+        <v>38</v>
+      </c>
+      <c r="O284" t="s">
+        <v>38</v>
+      </c>
+      <c r="P284" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q284" t="s">
+        <v>39</v>
+      </c>
+      <c r="R284" t="s">
+        <v>39</v>
+      </c>
+      <c r="S284" t="s">
+        <v>39</v>
+      </c>
+      <c r="T284" t="s">
+        <v>1173</v>
+      </c>
+      <c r="U284" t="s">
+        <v>39</v>
+      </c>
+      <c r="V284"/>
+      <c r="W284"/>
+      <c r="X284"/>
+      <c r="Y284"/>
+      <c r="Z284"/>
+      <c r="AA284"/>
+      <c r="AB284"/>
+      <c r="AC284">
+        <v>0.0</v>
+      </c>
+      <c r="AD284">
+        <v>12312355555.0</v>
+      </c>
+      <c r="AE284">
+        <v>12312355555.0</v>
+      </c>
+    </row>
+    <row r="285" spans="1:31">
+      <c r="A285">
+        <v>284</v>
+      </c>
+      <c r="B285" t="s">
+        <v>1174</v>
+      </c>
+      <c r="C285" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D285" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E285" t="s">
+        <v>1177</v>
+      </c>
+      <c r="F285" t="s">
+        <v>35</v>
+      </c>
+      <c r="G285"/>
+      <c r="H285" t="s">
+        <v>1137</v>
+      </c>
+      <c r="I285" t="s">
+        <v>35</v>
+      </c>
+      <c r="J285" t="s">
+        <v>54</v>
+      </c>
+      <c r="K285" t="s">
+        <v>38</v>
+      </c>
+      <c r="L285" t="s">
+        <v>38</v>
+      </c>
+      <c r="M285" t="s">
+        <v>38</v>
+      </c>
+      <c r="N285" t="s">
+        <v>38</v>
+      </c>
+      <c r="O285" t="s">
+        <v>38</v>
+      </c>
+      <c r="P285" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q285" t="s">
+        <v>39</v>
+      </c>
+      <c r="R285" t="s">
+        <v>39</v>
+      </c>
+      <c r="S285" t="s">
+        <v>39</v>
+      </c>
+      <c r="T285" t="s">
+        <v>1143</v>
+      </c>
+      <c r="U285" t="s">
+        <v>39</v>
+      </c>
+      <c r="V285"/>
+      <c r="W285"/>
+      <c r="X285"/>
+      <c r="Y285"/>
+      <c r="Z285"/>
+      <c r="AA285"/>
+      <c r="AB285"/>
+      <c r="AC285">
+        <v>0.0</v>
+      </c>
+      <c r="AD285">
+        <v>55555.0</v>
+      </c>
+      <c r="AE285">
+        <v>55555.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>